<commit_message>
Updated the .NET and Docker to .NET 10
</commit_message>
<xml_diff>
--- a/Files/rentRollDetails.xlsx
+++ b/Files/rentRollDetails.xlsx
@@ -684,7 +684,7 @@
       <font/>
       <fill>
         <patternFill>
-          <fgColor rgb="FF9C0055"/>
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
@@ -971,7 +971,7 @@
         <v>47118</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H2">
         <v>3217</v>

</xml_diff>